<commit_message>
regenerate derived taxonomy artifacts
</commit_message>
<xml_diff>
--- a/crosswalk/FT3-F3-crosswalk.xlsx
+++ b/crosswalk/FT3-F3-crosswalk.xlsx
@@ -8,7 +8,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="320">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="327">
   <si>
     <t>ft3_id</t>
   </si>
@@ -148,7 +148,7 @@
     <t>Acquire Access: Botnet</t>
   </si>
   <si>
-    <t>derived</t>
+    <t>subset</t>
   </si>
   <si>
     <t>FT007.002</t>
@@ -253,9 +253,6 @@
     <t>Acquire Infrastructure</t>
   </si>
   <si>
-    <t>subset</t>
-  </si>
-  <si>
     <t>T1588</t>
   </si>
   <si>
@@ -310,6 +307,12 @@
     <t>Account Takeover: Exposed Credential</t>
   </si>
   <si>
+    <t>F1006.001</t>
+  </si>
+  <si>
+    <t>Account Takeover: Exposed API Key</t>
+  </si>
+  <si>
     <t>FT011.002</t>
   </si>
   <si>
@@ -664,6 +667,12 @@
     <t>Account Manipulation: Additional Authorized Account</t>
   </si>
   <si>
+    <t>F1005.002</t>
+  </si>
+  <si>
+    <t>Account Manipulation: Add Authorized User</t>
+  </si>
+  <si>
     <t>FT037.003</t>
   </si>
   <si>
@@ -733,7 +742,19 @@
     <t>Account Manipulation: Additional Payment Methods</t>
   </si>
   <si>
+    <t>F1005.006</t>
+  </si>
+  <si>
+    <t>Account Manipulation: Change of Payment Details</t>
+  </si>
+  <si>
     <t>FT042.002</t>
+  </si>
+  <si>
+    <t>F1005.001</t>
+  </si>
+  <si>
+    <t>Account Manipulation: Account Linking</t>
   </si>
   <si>
     <t>FT042.003</t>
@@ -1524,24 +1545,24 @@
         <v>80</v>
       </c>
       <c r="E33" t="s">
+        <v>46</v>
+      </c>
+      <c r="F33" t="s">
         <v>81</v>
-      </c>
-      <c r="F33" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s">
+        <v>82</v>
+      </c>
+      <c r="B34" t="s">
         <v>83</v>
       </c>
-      <c r="B34" t="s">
+      <c r="C34" t="s">
         <v>84</v>
       </c>
-      <c r="C34" t="s">
-        <v>85</v>
-      </c>
       <c r="D34" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E34" t="s">
         <v>9</v>
@@ -1552,36 +1573,36 @@
     </row>
     <row r="35">
       <c r="A35" t="s">
+        <v>85</v>
+      </c>
+      <c r="B35" t="s">
         <v>86</v>
       </c>
-      <c r="B35" t="s">
+      <c r="C35" t="s">
+        <v>84</v>
+      </c>
+      <c r="D35" t="s">
+        <v>83</v>
+      </c>
+      <c r="E35" t="s">
+        <v>46</v>
+      </c>
+      <c r="F35" t="s">
         <v>87</v>
-      </c>
-      <c r="C35" t="s">
-        <v>85</v>
-      </c>
-      <c r="D35" t="s">
-        <v>84</v>
-      </c>
-      <c r="E35" t="s">
-        <v>46</v>
-      </c>
-      <c r="F35" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s">
+        <v>88</v>
+      </c>
+      <c r="B36" t="s">
         <v>89</v>
       </c>
-      <c r="B36" t="s">
-        <v>90</v>
-      </c>
       <c r="C36" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D36" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E36" t="s">
         <v>46</v>
@@ -1592,56 +1613,56 @@
     </row>
     <row r="37">
       <c r="A37" t="s">
+        <v>90</v>
+      </c>
+      <c r="B37" t="s">
         <v>91</v>
       </c>
-      <c r="B37" t="s">
-        <v>92</v>
-      </c>
       <c r="C37" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D37" t="s">
+        <v>83</v>
+      </c>
+      <c r="E37" t="s">
+        <v>46</v>
+      </c>
+      <c r="F37" t="s">
         <v>84</v>
-      </c>
-      <c r="E37" t="s">
-        <v>46</v>
-      </c>
-      <c r="F37" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s">
+        <v>92</v>
+      </c>
+      <c r="B38" t="s">
         <v>93</v>
       </c>
-      <c r="B38" t="s">
-        <v>94</v>
-      </c>
       <c r="C38" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D38" t="s">
+        <v>83</v>
+      </c>
+      <c r="E38" t="s">
+        <v>46</v>
+      </c>
+      <c r="F38" t="s">
         <v>84</v>
-      </c>
-      <c r="E38" t="s">
-        <v>46</v>
-      </c>
-      <c r="F38" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s">
+        <v>94</v>
+      </c>
+      <c r="B39" t="s">
         <v>95</v>
       </c>
-      <c r="B39" t="s">
+      <c r="C39" t="s">
         <v>96</v>
       </c>
-      <c r="C39" t="s">
-        <v>97</v>
-      </c>
       <c r="D39" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E39" t="s">
         <v>9</v>
@@ -1649,16 +1670,16 @@
     </row>
     <row r="40">
       <c r="A40" t="s">
+        <v>97</v>
+      </c>
+      <c r="B40" t="s">
         <v>98</v>
       </c>
-      <c r="B40" t="s">
+      <c r="C40" t="s">
         <v>99</v>
       </c>
-      <c r="C40" t="s">
-        <v>97</v>
-      </c>
       <c r="D40" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="E40" t="s">
         <v>46</v>
@@ -1666,16 +1687,16 @@
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B41" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C41" t="s">
+        <v>103</v>
+      </c>
+      <c r="D41" t="s">
         <v>102</v>
-      </c>
-      <c r="D41" t="s">
-        <v>101</v>
       </c>
       <c r="E41" t="s">
         <v>9</v>
@@ -1683,16 +1704,16 @@
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B42" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C42" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D42" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E42" t="s">
         <v>46</v>
@@ -1700,16 +1721,16 @@
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B43" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C43" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D43" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E43" t="s">
         <v>46</v>
@@ -1717,16 +1738,16 @@
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B44" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C44" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D44" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E44" t="s">
         <v>46</v>
@@ -1734,16 +1755,16 @@
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B45" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C45" t="s">
+        <v>112</v>
+      </c>
+      <c r="D45" t="s">
         <v>111</v>
-      </c>
-      <c r="D45" t="s">
-        <v>110</v>
       </c>
       <c r="E45" t="s">
         <v>9</v>
@@ -1751,16 +1772,16 @@
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B46" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C46" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D46" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E46" t="s">
         <v>9</v>
@@ -1768,10 +1789,10 @@
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B47" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E47" t="s">
         <v>12</v>
@@ -1779,30 +1800,30 @@
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B48" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C48" t="s">
+        <v>121</v>
+      </c>
+      <c r="D48" t="s">
         <v>120</v>
-      </c>
-      <c r="D48" t="s">
-        <v>119</v>
       </c>
       <c r="E48" t="s">
         <v>9</v>
       </c>
       <c r="F48" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B49" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E49" t="s">
         <v>12</v>
@@ -1810,110 +1831,110 @@
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B50" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C50" t="s">
+        <v>126</v>
+      </c>
+      <c r="D50" t="s">
         <v>125</v>
-      </c>
-      <c r="D50" t="s">
-        <v>124</v>
       </c>
       <c r="E50" t="s">
         <v>9</v>
       </c>
       <c r="F50" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="s">
+        <v>127</v>
+      </c>
+      <c r="B51" t="s">
+        <v>128</v>
+      </c>
+      <c r="C51" t="s">
         <v>126</v>
       </c>
-      <c r="B51" t="s">
-        <v>127</v>
-      </c>
-      <c r="C51" t="s">
+      <c r="D51" t="s">
         <v>125</v>
       </c>
-      <c r="D51" t="s">
-        <v>124</v>
-      </c>
       <c r="E51" t="s">
         <v>46</v>
       </c>
       <c r="F51" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B52" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C52" t="s">
+        <v>126</v>
+      </c>
+      <c r="D52" t="s">
         <v>125</v>
       </c>
-      <c r="D52" t="s">
-        <v>124</v>
-      </c>
       <c r="E52" t="s">
         <v>46</v>
       </c>
       <c r="F52" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B53" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C53" t="s">
+        <v>126</v>
+      </c>
+      <c r="D53" t="s">
         <v>125</v>
       </c>
-      <c r="D53" t="s">
-        <v>124</v>
-      </c>
       <c r="E53" t="s">
         <v>46</v>
       </c>
       <c r="F53" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B54" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C54" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D54" t="s">
+        <v>136</v>
+      </c>
+      <c r="E54" t="s">
+        <v>46</v>
+      </c>
+      <c r="F54" t="s">
         <v>135</v>
-      </c>
-      <c r="E54" t="s">
-        <v>81</v>
-      </c>
-      <c r="F54" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B55" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="E55" t="s">
         <v>12</v>
@@ -1921,16 +1942,16 @@
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B56" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C56" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D56" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="E56" t="s">
         <v>9</v>
@@ -1938,27 +1959,27 @@
     </row>
     <row r="57">
       <c r="A57" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B57" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C57" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D57" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E57" t="s">
-        <v>81</v>
+        <v>46</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B58" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E58" t="s">
         <v>12</v>
@@ -1966,16 +1987,16 @@
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B59" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C59" t="s">
+        <v>151</v>
+      </c>
+      <c r="D59" t="s">
         <v>150</v>
-      </c>
-      <c r="D59" t="s">
-        <v>149</v>
       </c>
       <c r="E59" t="s">
         <v>9</v>
@@ -1983,10 +2004,10 @@
     </row>
     <row r="60">
       <c r="A60" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B60" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="E60" t="s">
         <v>12</v>
@@ -1994,27 +2015,27 @@
     </row>
     <row r="61">
       <c r="A61" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B61" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C61" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D61" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E61" t="s">
-        <v>81</v>
+        <v>46</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B62" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E62" t="s">
         <v>12</v>
@@ -2022,16 +2043,16 @@
     </row>
     <row r="63">
       <c r="A63" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B63" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C63" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D63" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E63" t="s">
         <v>9</v>
@@ -2039,95 +2060,95 @@
     </row>
     <row r="64">
       <c r="A64" t="s">
+        <v>164</v>
+      </c>
+      <c r="B64" t="s">
+        <v>165</v>
+      </c>
+      <c r="C64" t="s">
+        <v>162</v>
+      </c>
+      <c r="D64" t="s">
         <v>163</v>
       </c>
-      <c r="B64" t="s">
-        <v>164</v>
-      </c>
-      <c r="C64" t="s">
-        <v>161</v>
-      </c>
-      <c r="D64" t="s">
-        <v>162</v>
-      </c>
       <c r="E64" t="s">
-        <v>81</v>
+        <v>46</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B65" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C65" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D65" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E65" t="s">
-        <v>81</v>
+        <v>46</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B66" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C66" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D66" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E66" t="s">
-        <v>81</v>
+        <v>46</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B67" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C67" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D67" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E67" t="s">
-        <v>81</v>
+        <v>46</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B68" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C68" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D68" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E68" t="s">
-        <v>81</v>
+        <v>46</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B69" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="E69" t="s">
         <v>12</v>
@@ -2135,10 +2156,10 @@
     </row>
     <row r="70">
       <c r="A70" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B70" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="E70" t="s">
         <v>12</v>
@@ -2146,10 +2167,10 @@
     </row>
     <row r="71">
       <c r="A71" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B71" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="E71" t="s">
         <v>12</v>
@@ -2157,10 +2178,10 @@
     </row>
     <row r="72">
       <c r="A72" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B72" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="E72" t="s">
         <v>12</v>
@@ -2168,30 +2189,30 @@
     </row>
     <row r="73">
       <c r="A73" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B73" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="C73" t="s">
+        <v>126</v>
+      </c>
+      <c r="D73" t="s">
         <v>125</v>
       </c>
-      <c r="D73" t="s">
-        <v>124</v>
-      </c>
       <c r="E73" t="s">
         <v>46</v>
       </c>
       <c r="F73" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B74" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="E74" t="s">
         <v>12</v>
@@ -2199,16 +2220,16 @@
     </row>
     <row r="75">
       <c r="A75" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B75" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="C75" t="s">
+        <v>188</v>
+      </c>
+      <c r="D75" t="s">
         <v>187</v>
-      </c>
-      <c r="D75" t="s">
-        <v>186</v>
       </c>
       <c r="E75" t="s">
         <v>9</v>
@@ -2216,16 +2237,16 @@
     </row>
     <row r="76">
       <c r="A76" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B76" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C76" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="D76" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E76" t="s">
         <v>9</v>
@@ -2233,10 +2254,10 @@
     </row>
     <row r="77">
       <c r="A77" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B77" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="E77" t="s">
         <v>12</v>
@@ -2244,16 +2265,16 @@
     </row>
     <row r="78">
       <c r="A78" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B78" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C78" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D78" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E78" t="s">
         <v>9</v>
@@ -2261,10 +2282,10 @@
     </row>
     <row r="79">
       <c r="A79" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B79" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="E79" t="s">
         <v>12</v>
@@ -2272,10 +2293,10 @@
     </row>
     <row r="80">
       <c r="A80" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B80" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="E80" t="s">
         <v>12</v>
@@ -2283,10 +2304,10 @@
     </row>
     <row r="81">
       <c r="A81" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B81" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="E81" t="s">
         <v>12</v>
@@ -2294,10 +2315,10 @@
     </row>
     <row r="82">
       <c r="A82" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B82" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="E82" t="s">
         <v>12</v>
@@ -2305,27 +2326,27 @@
     </row>
     <row r="83">
       <c r="A83" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B83" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="C83" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D83" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E83" t="s">
-        <v>81</v>
+        <v>46</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B84" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="E84" t="s">
         <v>12</v>
@@ -2333,10 +2354,10 @@
     </row>
     <row r="85">
       <c r="A85" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B85" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="E85" t="s">
         <v>12</v>
@@ -2344,10 +2365,10 @@
     </row>
     <row r="86">
       <c r="A86" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B86" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="E86" t="s">
         <v>12</v>
@@ -2355,16 +2376,16 @@
     </row>
     <row r="87">
       <c r="A87" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B87" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C87" t="s">
+        <v>214</v>
+      </c>
+      <c r="D87" t="s">
         <v>213</v>
-      </c>
-      <c r="D87" t="s">
-        <v>212</v>
       </c>
       <c r="E87" t="s">
         <v>9</v>
@@ -2372,16 +2393,16 @@
     </row>
     <row r="88">
       <c r="A88" t="s">
+        <v>215</v>
+      </c>
+      <c r="B88" t="s">
+        <v>216</v>
+      </c>
+      <c r="C88" t="s">
         <v>214</v>
       </c>
-      <c r="B88" t="s">
-        <v>215</v>
-      </c>
-      <c r="C88" t="s">
+      <c r="D88" t="s">
         <v>213</v>
-      </c>
-      <c r="D88" t="s">
-        <v>212</v>
       </c>
       <c r="E88" t="s">
         <v>46</v>
@@ -2389,16 +2410,16 @@
     </row>
     <row r="89">
       <c r="A89" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B89" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C89" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="D89" t="s">
-        <v>212</v>
+        <v>220</v>
       </c>
       <c r="E89" t="s">
         <v>46</v>
@@ -2406,16 +2427,16 @@
     </row>
     <row r="90">
       <c r="A90" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="B90" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="C90" t="s">
+        <v>214</v>
+      </c>
+      <c r="D90" t="s">
         <v>213</v>
-      </c>
-      <c r="D90" t="s">
-        <v>212</v>
       </c>
       <c r="E90" t="s">
         <v>46</v>
@@ -2423,10 +2444,10 @@
     </row>
     <row r="91">
       <c r="A91" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="B91" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="E91" t="s">
         <v>12</v>
@@ -2434,10 +2455,10 @@
     </row>
     <row r="92">
       <c r="A92" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="B92" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="E92" t="s">
         <v>12</v>
@@ -2445,10 +2466,10 @@
     </row>
     <row r="93">
       <c r="A93" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="B93" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="E93" t="s">
         <v>12</v>
@@ -2456,10 +2477,10 @@
     </row>
     <row r="94">
       <c r="A94" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="B94" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="E94" t="s">
         <v>12</v>
@@ -2467,10 +2488,10 @@
     </row>
     <row r="95">
       <c r="A95" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="B95" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="E95" t="s">
         <v>12</v>
@@ -2478,10 +2499,10 @@
     </row>
     <row r="96">
       <c r="A96" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="B96" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="E96" t="s">
         <v>12</v>
@@ -2489,10 +2510,10 @@
     </row>
     <row r="97">
       <c r="A97" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="B97" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="E97" t="s">
         <v>12</v>
@@ -2500,10 +2521,10 @@
     </row>
     <row r="98">
       <c r="A98" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="B98" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="E98" t="s">
         <v>12</v>
@@ -2511,10 +2532,10 @@
     </row>
     <row r="99">
       <c r="A99" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="B99" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="E99" t="s">
         <v>12</v>
@@ -2522,16 +2543,16 @@
     </row>
     <row r="100">
       <c r="A100" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="B100" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C100" t="s">
+        <v>214</v>
+      </c>
+      <c r="D100" t="s">
         <v>213</v>
-      </c>
-      <c r="D100" t="s">
-        <v>212</v>
       </c>
       <c r="E100" t="s">
         <v>9</v>
@@ -2539,16 +2560,16 @@
     </row>
     <row r="101">
       <c r="A101" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="B101" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="C101" t="s">
-        <v>213</v>
+        <v>244</v>
       </c>
       <c r="D101" t="s">
-        <v>212</v>
+        <v>245</v>
       </c>
       <c r="E101" t="s">
         <v>46</v>
@@ -2556,16 +2577,16 @@
     </row>
     <row r="102">
       <c r="A102" t="s">
-        <v>241</v>
+        <v>246</v>
       </c>
       <c r="B102" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="C102" t="s">
-        <v>213</v>
+        <v>247</v>
       </c>
       <c r="D102" t="s">
-        <v>212</v>
+        <v>248</v>
       </c>
       <c r="E102" t="s">
         <v>46</v>
@@ -2573,16 +2594,16 @@
     </row>
     <row r="103">
       <c r="A103" t="s">
-        <v>242</v>
+        <v>249</v>
       </c>
       <c r="B103" t="s">
-        <v>243</v>
+        <v>250</v>
       </c>
       <c r="C103" t="s">
+        <v>214</v>
+      </c>
+      <c r="D103" t="s">
         <v>213</v>
-      </c>
-      <c r="D103" t="s">
-        <v>212</v>
       </c>
       <c r="E103" t="s">
         <v>46</v>
@@ -2590,16 +2611,16 @@
     </row>
     <row r="104">
       <c r="A104" t="s">
-        <v>244</v>
+        <v>251</v>
       </c>
       <c r="B104" t="s">
-        <v>245</v>
+        <v>252</v>
       </c>
       <c r="C104" t="s">
+        <v>214</v>
+      </c>
+      <c r="D104" t="s">
         <v>213</v>
-      </c>
-      <c r="D104" t="s">
-        <v>212</v>
       </c>
       <c r="E104" t="s">
         <v>46</v>
@@ -2607,16 +2628,16 @@
     </row>
     <row r="105">
       <c r="A105" t="s">
-        <v>246</v>
+        <v>253</v>
       </c>
       <c r="B105" t="s">
-        <v>247</v>
+        <v>254</v>
       </c>
       <c r="C105" t="s">
-        <v>213</v>
+        <v>244</v>
       </c>
       <c r="D105" t="s">
-        <v>212</v>
+        <v>245</v>
       </c>
       <c r="E105" t="s">
         <v>46</v>
@@ -2624,16 +2645,16 @@
     </row>
     <row r="106">
       <c r="A106" t="s">
+        <v>255</v>
+      </c>
+      <c r="B106" t="s">
+        <v>256</v>
+      </c>
+      <c r="C106" t="s">
+        <v>247</v>
+      </c>
+      <c r="D106" t="s">
         <v>248</v>
-      </c>
-      <c r="B106" t="s">
-        <v>249</v>
-      </c>
-      <c r="C106" t="s">
-        <v>213</v>
-      </c>
-      <c r="D106" t="s">
-        <v>212</v>
       </c>
       <c r="E106" t="s">
         <v>46</v>
@@ -2641,16 +2662,16 @@
     </row>
     <row r="107">
       <c r="A107" t="s">
-        <v>250</v>
+        <v>257</v>
       </c>
       <c r="B107" t="s">
-        <v>251</v>
+        <v>258</v>
       </c>
       <c r="C107" t="s">
-        <v>252</v>
+        <v>259</v>
       </c>
       <c r="D107" t="s">
-        <v>251</v>
+        <v>258</v>
       </c>
       <c r="E107" t="s">
         <v>9</v>
@@ -2658,16 +2679,16 @@
     </row>
     <row r="108">
       <c r="A108" t="s">
-        <v>253</v>
+        <v>260</v>
       </c>
       <c r="B108" t="s">
-        <v>254</v>
+        <v>261</v>
       </c>
       <c r="C108" t="s">
+        <v>214</v>
+      </c>
+      <c r="D108" t="s">
         <v>213</v>
-      </c>
-      <c r="D108" t="s">
-        <v>212</v>
       </c>
       <c r="E108" t="s">
         <v>46</v>
@@ -2675,16 +2696,16 @@
     </row>
     <row r="109">
       <c r="A109" t="s">
-        <v>255</v>
+        <v>262</v>
       </c>
       <c r="B109" t="s">
-        <v>256</v>
+        <v>263</v>
       </c>
       <c r="C109" t="s">
-        <v>257</v>
+        <v>264</v>
       </c>
       <c r="D109" t="s">
-        <v>256</v>
+        <v>263</v>
       </c>
       <c r="E109" t="s">
         <v>9</v>
@@ -2692,10 +2713,10 @@
     </row>
     <row r="110">
       <c r="A110" t="s">
-        <v>258</v>
+        <v>265</v>
       </c>
       <c r="B110" t="s">
-        <v>259</v>
+        <v>266</v>
       </c>
       <c r="E110" t="s">
         <v>12</v>
@@ -2703,10 +2724,10 @@
     </row>
     <row r="111">
       <c r="A111" t="s">
-        <v>260</v>
+        <v>267</v>
       </c>
       <c r="B111" t="s">
-        <v>261</v>
+        <v>268</v>
       </c>
       <c r="E111" t="s">
         <v>12</v>
@@ -2714,10 +2735,10 @@
     </row>
     <row r="112">
       <c r="A112" t="s">
-        <v>262</v>
+        <v>269</v>
       </c>
       <c r="B112" t="s">
-        <v>263</v>
+        <v>270</v>
       </c>
       <c r="E112" t="s">
         <v>12</v>
@@ -2725,10 +2746,10 @@
     </row>
     <row r="113">
       <c r="A113" t="s">
-        <v>264</v>
+        <v>271</v>
       </c>
       <c r="B113" t="s">
-        <v>265</v>
+        <v>272</v>
       </c>
       <c r="E113" t="s">
         <v>12</v>
@@ -2736,36 +2757,36 @@
     </row>
     <row r="114">
       <c r="A114" t="s">
-        <v>266</v>
+        <v>273</v>
       </c>
       <c r="B114" t="s">
-        <v>267</v>
+        <v>274</v>
       </c>
       <c r="C114" t="s">
-        <v>268</v>
+        <v>275</v>
       </c>
       <c r="D114" t="s">
-        <v>267</v>
+        <v>274</v>
       </c>
       <c r="E114" t="s">
         <v>9</v>
       </c>
       <c r="F114" t="s">
-        <v>268</v>
+        <v>275</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="s">
-        <v>269</v>
+        <v>276</v>
       </c>
       <c r="B115" t="s">
-        <v>270</v>
+        <v>277</v>
       </c>
       <c r="C115" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D115" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E115" t="s">
         <v>9</v>
@@ -2773,10 +2794,10 @@
     </row>
     <row r="116">
       <c r="A116" t="s">
-        <v>271</v>
+        <v>278</v>
       </c>
       <c r="B116" t="s">
-        <v>272</v>
+        <v>279</v>
       </c>
       <c r="E116" t="s">
         <v>12</v>
@@ -2784,16 +2805,16 @@
     </row>
     <row r="117">
       <c r="A117" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="B117" t="s">
-        <v>274</v>
+        <v>281</v>
       </c>
       <c r="C117" t="s">
-        <v>275</v>
+        <v>282</v>
       </c>
       <c r="D117" t="s">
-        <v>276</v>
+        <v>283</v>
       </c>
       <c r="E117" t="s">
         <v>9</v>
@@ -2801,84 +2822,84 @@
     </row>
     <row r="118">
       <c r="A118" t="s">
-        <v>277</v>
+        <v>284</v>
       </c>
       <c r="B118" t="s">
-        <v>278</v>
+        <v>285</v>
       </c>
       <c r="C118" t="s">
-        <v>275</v>
+        <v>282</v>
       </c>
       <c r="D118" t="s">
-        <v>276</v>
+        <v>283</v>
       </c>
       <c r="E118" t="s">
-        <v>81</v>
+        <v>46</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="s">
-        <v>279</v>
+        <v>286</v>
       </c>
       <c r="B119" t="s">
-        <v>280</v>
+        <v>287</v>
       </c>
       <c r="C119" t="s">
-        <v>275</v>
+        <v>282</v>
       </c>
       <c r="D119" t="s">
-        <v>276</v>
+        <v>283</v>
       </c>
       <c r="E119" t="s">
-        <v>81</v>
+        <v>46</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="s">
-        <v>281</v>
+        <v>288</v>
       </c>
       <c r="B120" t="s">
+        <v>289</v>
+      </c>
+      <c r="C120" t="s">
         <v>282</v>
       </c>
-      <c r="C120" t="s">
-        <v>275</v>
-      </c>
       <c r="D120" t="s">
-        <v>276</v>
+        <v>283</v>
       </c>
       <c r="E120" t="s">
-        <v>81</v>
+        <v>46</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="s">
+        <v>290</v>
+      </c>
+      <c r="B121" t="s">
+        <v>291</v>
+      </c>
+      <c r="C121" t="s">
+        <v>282</v>
+      </c>
+      <c r="D121" t="s">
         <v>283</v>
       </c>
-      <c r="B121" t="s">
-        <v>284</v>
-      </c>
-      <c r="C121" t="s">
-        <v>275</v>
-      </c>
-      <c r="D121" t="s">
-        <v>276</v>
-      </c>
       <c r="E121" t="s">
-        <v>81</v>
+        <v>46</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="s">
-        <v>285</v>
+        <v>292</v>
       </c>
       <c r="B122" t="s">
-        <v>286</v>
+        <v>293</v>
       </c>
       <c r="C122" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D122" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E122" t="s">
         <v>9</v>
@@ -2886,169 +2907,169 @@
     </row>
     <row r="123">
       <c r="A123" t="s">
-        <v>287</v>
+        <v>294</v>
       </c>
       <c r="B123" t="s">
-        <v>288</v>
+        <v>295</v>
       </c>
       <c r="C123" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D123" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E123" t="s">
-        <v>81</v>
+        <v>46</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="s">
-        <v>289</v>
+        <v>296</v>
       </c>
       <c r="B124" t="s">
-        <v>290</v>
+        <v>297</v>
       </c>
       <c r="C124" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D124" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E124" t="s">
-        <v>81</v>
+        <v>46</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="B125" t="s">
-        <v>292</v>
+        <v>299</v>
       </c>
       <c r="C125" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D125" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E125" t="s">
-        <v>81</v>
+        <v>46</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="s">
-        <v>293</v>
+        <v>300</v>
       </c>
       <c r="B126" t="s">
-        <v>294</v>
+        <v>301</v>
       </c>
       <c r="C126" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D126" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E126" t="s">
-        <v>81</v>
+        <v>46</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="s">
-        <v>295</v>
+        <v>302</v>
       </c>
       <c r="B127" t="s">
-        <v>296</v>
+        <v>303</v>
       </c>
       <c r="C127" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D127" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E127" t="s">
-        <v>81</v>
+        <v>46</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="s">
-        <v>297</v>
+        <v>304</v>
       </c>
       <c r="B128" t="s">
-        <v>298</v>
+        <v>305</v>
       </c>
       <c r="C128" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D128" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E128" t="s">
-        <v>81</v>
+        <v>46</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="s">
-        <v>299</v>
+        <v>306</v>
       </c>
       <c r="B129" t="s">
-        <v>300</v>
+        <v>307</v>
       </c>
       <c r="C129" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D129" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E129" t="s">
-        <v>81</v>
+        <v>46</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="s">
-        <v>301</v>
+        <v>308</v>
       </c>
       <c r="B130" t="s">
-        <v>302</v>
+        <v>309</v>
       </c>
       <c r="C130" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D130" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E130" t="s">
-        <v>81</v>
+        <v>46</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="s">
-        <v>303</v>
+        <v>310</v>
       </c>
       <c r="B131" t="s">
-        <v>304</v>
+        <v>311</v>
       </c>
       <c r="C131" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D131" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E131" t="s">
-        <v>81</v>
+        <v>46</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="s">
-        <v>305</v>
+        <v>312</v>
       </c>
       <c r="B132" t="s">
-        <v>306</v>
+        <v>313</v>
       </c>
       <c r="C132" t="s">
-        <v>307</v>
+        <v>314</v>
       </c>
       <c r="D132" t="s">
-        <v>306</v>
+        <v>313</v>
       </c>
       <c r="E132" t="s">
         <v>9</v>
@@ -3056,16 +3077,16 @@
     </row>
     <row r="133">
       <c r="A133" t="s">
-        <v>308</v>
+        <v>315</v>
       </c>
       <c r="B133" t="s">
-        <v>309</v>
+        <v>316</v>
       </c>
       <c r="C133" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D133" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="E133" t="s">
         <v>9</v>
@@ -3073,27 +3094,27 @@
     </row>
     <row r="134">
       <c r="A134" t="s">
-        <v>310</v>
+        <v>317</v>
       </c>
       <c r="B134" t="s">
-        <v>311</v>
+        <v>318</v>
       </c>
       <c r="C134" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D134" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="E134" t="s">
-        <v>81</v>
+        <v>46</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="s">
-        <v>312</v>
+        <v>319</v>
       </c>
       <c r="B135" t="s">
-        <v>313</v>
+        <v>320</v>
       </c>
       <c r="E135" t="s">
         <v>12</v>
@@ -3101,10 +3122,10 @@
     </row>
     <row r="136">
       <c r="A136" t="s">
-        <v>314</v>
+        <v>321</v>
       </c>
       <c r="B136" t="s">
-        <v>315</v>
+        <v>322</v>
       </c>
       <c r="E136" t="s">
         <v>12</v>
@@ -3112,10 +3133,10 @@
     </row>
     <row r="137">
       <c r="A137" t="s">
-        <v>316</v>
+        <v>323</v>
       </c>
       <c r="B137" t="s">
-        <v>317</v>
+        <v>324</v>
       </c>
       <c r="E137" t="s">
         <v>12</v>
@@ -3123,10 +3144,10 @@
     </row>
     <row r="138">
       <c r="A138" t="s">
-        <v>318</v>
+        <v>325</v>
       </c>
       <c r="B138" t="s">
-        <v>319</v>
+        <v>326</v>
       </c>
       <c r="E138" t="s">
         <v>12</v>

</xml_diff>

<commit_message>
Refresh generated derivation artifacts
</commit_message>
<xml_diff>
--- a/crosswalk/FT3-F3-crosswalk.xlsx
+++ b/crosswalk/FT3-F3-crosswalk.xlsx
@@ -8,7 +8,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="320">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="337" uniqueCount="337">
   <si>
     <t>ft3_id</t>
   </si>
@@ -406,6 +406,21 @@
     <t>Phishing: Backup Code</t>
   </si>
   <si>
+    <t>FT016.004</t>
+  </si>
+  <si>
+    <t>Phishing: Real-Time OTP Relay via Operator-Controlled Phishing Kit</t>
+  </si>
+  <si>
+    <t>T1111</t>
+  </si>
+  <si>
+    <t>Multi-Factor Authentication Interception</t>
+  </si>
+  <si>
+    <t>partial</t>
+  </si>
+  <si>
     <t>FT017</t>
   </si>
   <si>
@@ -529,6 +544,12 @@
     <t>Falsifying Business Documents: Fake SS-4 Confirmation Letter</t>
   </si>
   <si>
+    <t>FT026.006</t>
+  </si>
+  <si>
+    <t>Falsifying Business Documents: Live-Source Tax Certificate Forgery</t>
+  </si>
+  <si>
     <t>FT027</t>
   </si>
   <si>
@@ -968,6 +989,36 @@
   </si>
   <si>
     <t>Card Holder Details Collection: Card Details</t>
+  </si>
+  <si>
+    <t>FT057</t>
+  </si>
+  <si>
+    <t>Voice Phishing (Vishing)</t>
+  </si>
+  <si>
+    <t>F1040</t>
+  </si>
+  <si>
+    <t>Phone Number Spoofing</t>
+  </si>
+  <si>
+    <t>FT058</t>
+  </si>
+  <si>
+    <t>ClickFix Run-Dialog Social Engineering</t>
+  </si>
+  <si>
+    <t>FT059</t>
+  </si>
+  <si>
+    <t>Mobile Banking Trojan Distribution and Device Takeover</t>
+  </si>
+  <si>
+    <t>T1453</t>
+  </si>
+  <si>
+    <t>Abuse Accessibility Features</t>
   </si>
 </sst>
 </file>
@@ -1902,7 +1953,7 @@
         <v>135</v>
       </c>
       <c r="E54" t="s">
-        <v>81</v>
+        <v>136</v>
       </c>
       <c r="F54" t="s">
         <v>134</v>
@@ -1910,162 +1961,165 @@
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B55" t="s">
-        <v>137</v>
+        <v>138</v>
+      </c>
+      <c r="C55" t="s">
+        <v>139</v>
+      </c>
+      <c r="D55" t="s">
+        <v>140</v>
       </c>
       <c r="E55" t="s">
-        <v>12</v>
+        <v>81</v>
+      </c>
+      <c r="F55" t="s">
+        <v>139</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="B56" t="s">
-        <v>139</v>
-      </c>
-      <c r="C56" t="s">
-        <v>140</v>
-      </c>
-      <c r="D56" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="E56" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B57" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C57" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D57" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E57" t="s">
-        <v>81</v>
+        <v>9</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B58" t="s">
-        <v>147</v>
+        <v>148</v>
+      </c>
+      <c r="C58" t="s">
+        <v>149</v>
+      </c>
+      <c r="D58" t="s">
+        <v>150</v>
       </c>
       <c r="E58" t="s">
-        <v>12</v>
+        <v>81</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="B59" t="s">
-        <v>149</v>
-      </c>
-      <c r="C59" t="s">
-        <v>150</v>
-      </c>
-      <c r="D59" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="E59" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B60" t="s">
-        <v>152</v>
+        <v>154</v>
+      </c>
+      <c r="C60" t="s">
+        <v>155</v>
+      </c>
+      <c r="D60" t="s">
+        <v>154</v>
       </c>
       <c r="E60" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="B61" t="s">
-        <v>154</v>
-      </c>
-      <c r="C61" t="s">
-        <v>155</v>
-      </c>
-      <c r="D61" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E61" t="s">
-        <v>81</v>
+        <v>12</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B62" t="s">
-        <v>158</v>
+        <v>159</v>
+      </c>
+      <c r="C62" t="s">
+        <v>160</v>
+      </c>
+      <c r="D62" t="s">
+        <v>161</v>
       </c>
       <c r="E62" t="s">
-        <v>12</v>
+        <v>81</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="B63" t="s">
-        <v>160</v>
-      </c>
-      <c r="C63" t="s">
-        <v>161</v>
-      </c>
-      <c r="D63" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E63" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B64" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C64" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="D64" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="E64" t="s">
-        <v>81</v>
+        <v>9</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="B65" t="s">
+        <v>169</v>
+      </c>
+      <c r="C65" t="s">
         <v>166</v>
       </c>
-      <c r="C65" t="s">
-        <v>161</v>
-      </c>
       <c r="D65" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="E65" t="s">
         <v>81</v>
@@ -2073,16 +2127,16 @@
     </row>
     <row r="66">
       <c r="A66" t="s">
+        <v>170</v>
+      </c>
+      <c r="B66" t="s">
+        <v>171</v>
+      </c>
+      <c r="C66" t="s">
+        <v>166</v>
+      </c>
+      <c r="D66" t="s">
         <v>167</v>
-      </c>
-      <c r="B66" t="s">
-        <v>168</v>
-      </c>
-      <c r="C66" t="s">
-        <v>161</v>
-      </c>
-      <c r="D66" t="s">
-        <v>162</v>
       </c>
       <c r="E66" t="s">
         <v>81</v>
@@ -2090,16 +2144,16 @@
     </row>
     <row r="67">
       <c r="A67" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="B67" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="C67" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="D67" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="E67" t="s">
         <v>81</v>
@@ -2107,16 +2161,16 @@
     </row>
     <row r="68">
       <c r="A68" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="B68" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="C68" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="D68" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="E68" t="s">
         <v>81</v>
@@ -2124,32 +2178,44 @@
     </row>
     <row r="69">
       <c r="A69" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="B69" t="s">
-        <v>174</v>
+        <v>177</v>
+      </c>
+      <c r="C69" t="s">
+        <v>166</v>
+      </c>
+      <c r="D69" t="s">
+        <v>167</v>
       </c>
       <c r="E69" t="s">
-        <v>12</v>
+        <v>81</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="B70" t="s">
-        <v>176</v>
+        <v>179</v>
+      </c>
+      <c r="C70" t="s">
+        <v>166</v>
+      </c>
+      <c r="D70" t="s">
+        <v>167</v>
       </c>
       <c r="E70" t="s">
-        <v>12</v>
+        <v>81</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="B71" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="E71" t="s">
         <v>12</v>
@@ -2157,10 +2223,10 @@
     </row>
     <row r="72">
       <c r="A72" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="B72" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="E72" t="s">
         <v>12</v>
@@ -2168,30 +2234,21 @@
     </row>
     <row r="73">
       <c r="A73" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="B73" t="s">
-        <v>182</v>
-      </c>
-      <c r="C73" t="s">
-        <v>125</v>
-      </c>
-      <c r="D73" t="s">
-        <v>124</v>
+        <v>185</v>
       </c>
       <c r="E73" t="s">
-        <v>46</v>
-      </c>
-      <c r="F73" t="s">
-        <v>125</v>
+        <v>12</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="B74" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="E74" t="s">
         <v>12</v>
@@ -2199,36 +2256,33 @@
     </row>
     <row r="75">
       <c r="A75" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="B75" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="C75" t="s">
-        <v>187</v>
+        <v>125</v>
       </c>
       <c r="D75" t="s">
-        <v>186</v>
+        <v>124</v>
       </c>
       <c r="E75" t="s">
-        <v>9</v>
+        <v>46</v>
+      </c>
+      <c r="F75" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B76" t="s">
-        <v>189</v>
-      </c>
-      <c r="C76" t="s">
-        <v>190</v>
-      </c>
-      <c r="D76" t="s">
         <v>191</v>
       </c>
       <c r="E76" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="77">
@@ -2238,22 +2292,28 @@
       <c r="B77" t="s">
         <v>193</v>
       </c>
+      <c r="C77" t="s">
+        <v>194</v>
+      </c>
+      <c r="D77" t="s">
+        <v>193</v>
+      </c>
       <c r="E77" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B78" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C78" t="s">
-        <v>114</v>
+        <v>197</v>
       </c>
       <c r="D78" t="s">
-        <v>115</v>
+        <v>198</v>
       </c>
       <c r="E78" t="s">
         <v>9</v>
@@ -2261,10 +2321,10 @@
     </row>
     <row r="79">
       <c r="A79" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="B79" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="E79" t="s">
         <v>12</v>
@@ -2272,21 +2332,27 @@
     </row>
     <row r="80">
       <c r="A80" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="B80" t="s">
-        <v>199</v>
+        <v>202</v>
+      </c>
+      <c r="C80" t="s">
+        <v>114</v>
+      </c>
+      <c r="D80" t="s">
+        <v>115</v>
       </c>
       <c r="E80" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="B81" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="E81" t="s">
         <v>12</v>
@@ -2294,10 +2360,10 @@
     </row>
     <row r="82">
       <c r="A82" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="B82" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="E82" t="s">
         <v>12</v>
@@ -2305,27 +2371,21 @@
     </row>
     <row r="83">
       <c r="A83" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="B83" t="s">
-        <v>205</v>
-      </c>
-      <c r="C83" t="s">
-        <v>155</v>
-      </c>
-      <c r="D83" t="s">
-        <v>156</v>
+        <v>208</v>
       </c>
       <c r="E83" t="s">
-        <v>81</v>
+        <v>12</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B84" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="E84" t="s">
         <v>12</v>
@@ -2333,21 +2393,27 @@
     </row>
     <row r="85">
       <c r="A85" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="B85" t="s">
-        <v>152</v>
+        <v>212</v>
+      </c>
+      <c r="C85" t="s">
+        <v>160</v>
+      </c>
+      <c r="D85" t="s">
+        <v>161</v>
       </c>
       <c r="E85" t="s">
-        <v>12</v>
+        <v>81</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="B86" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="E86" t="s">
         <v>12</v>
@@ -2355,67 +2421,55 @@
     </row>
     <row r="87">
       <c r="A87" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="B87" t="s">
-        <v>212</v>
-      </c>
-      <c r="C87" t="s">
-        <v>213</v>
-      </c>
-      <c r="D87" t="s">
-        <v>212</v>
+        <v>157</v>
       </c>
       <c r="E87" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B88" t="s">
-        <v>215</v>
-      </c>
-      <c r="C88" t="s">
-        <v>213</v>
-      </c>
-      <c r="D88" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="E88" t="s">
-        <v>46</v>
+        <v>12</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B89" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="C89" t="s">
-        <v>213</v>
+        <v>220</v>
       </c>
       <c r="D89" t="s">
-        <v>212</v>
+        <v>219</v>
       </c>
       <c r="E89" t="s">
-        <v>46</v>
+        <v>9</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="B90" t="s">
+        <v>222</v>
+      </c>
+      <c r="C90" t="s">
+        <v>220</v>
+      </c>
+      <c r="D90" t="s">
         <v>219</v>
-      </c>
-      <c r="C90" t="s">
-        <v>213</v>
-      </c>
-      <c r="D90" t="s">
-        <v>212</v>
       </c>
       <c r="E90" t="s">
         <v>46</v>
@@ -2423,32 +2477,44 @@
     </row>
     <row r="91">
       <c r="A91" t="s">
+        <v>223</v>
+      </c>
+      <c r="B91" t="s">
+        <v>224</v>
+      </c>
+      <c r="C91" t="s">
         <v>220</v>
       </c>
-      <c r="B91" t="s">
-        <v>221</v>
+      <c r="D91" t="s">
+        <v>219</v>
       </c>
       <c r="E91" t="s">
-        <v>12</v>
+        <v>46</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="B92" t="s">
-        <v>223</v>
+        <v>226</v>
+      </c>
+      <c r="C92" t="s">
+        <v>220</v>
+      </c>
+      <c r="D92" t="s">
+        <v>219</v>
       </c>
       <c r="E92" t="s">
-        <v>12</v>
+        <v>46</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="B93" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="E93" t="s">
         <v>12</v>
@@ -2456,10 +2522,10 @@
     </row>
     <row r="94">
       <c r="A94" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="B94" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="E94" t="s">
         <v>12</v>
@@ -2467,10 +2533,10 @@
     </row>
     <row r="95">
       <c r="A95" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="B95" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="E95" t="s">
         <v>12</v>
@@ -2478,10 +2544,10 @@
     </row>
     <row r="96">
       <c r="A96" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="B96" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="E96" t="s">
         <v>12</v>
@@ -2489,10 +2555,10 @@
     </row>
     <row r="97">
       <c r="A97" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="B97" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="E97" t="s">
         <v>12</v>
@@ -2500,10 +2566,10 @@
     </row>
     <row r="98">
       <c r="A98" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="B98" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="E98" t="s">
         <v>12</v>
@@ -2511,10 +2577,10 @@
     </row>
     <row r="99">
       <c r="A99" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="B99" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="E99" t="s">
         <v>12</v>
@@ -2522,67 +2588,55 @@
     </row>
     <row r="100">
       <c r="A100" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="B100" t="s">
-        <v>212</v>
-      </c>
-      <c r="C100" t="s">
-        <v>213</v>
-      </c>
-      <c r="D100" t="s">
-        <v>212</v>
+        <v>242</v>
       </c>
       <c r="E100" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="B101" t="s">
-        <v>240</v>
-      </c>
-      <c r="C101" t="s">
-        <v>213</v>
-      </c>
-      <c r="D101" t="s">
-        <v>212</v>
+        <v>244</v>
       </c>
       <c r="E101" t="s">
-        <v>46</v>
+        <v>12</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="B102" t="s">
         <v>219</v>
       </c>
       <c r="C102" t="s">
-        <v>213</v>
+        <v>220</v>
       </c>
       <c r="D102" t="s">
-        <v>212</v>
+        <v>219</v>
       </c>
       <c r="E102" t="s">
-        <v>46</v>
+        <v>9</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="B103" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="C103" t="s">
-        <v>213</v>
+        <v>220</v>
       </c>
       <c r="D103" t="s">
-        <v>212</v>
+        <v>219</v>
       </c>
       <c r="E103" t="s">
         <v>46</v>
@@ -2590,16 +2644,16 @@
     </row>
     <row r="104">
       <c r="A104" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="B104" t="s">
-        <v>245</v>
+        <v>226</v>
       </c>
       <c r="C104" t="s">
-        <v>213</v>
+        <v>220</v>
       </c>
       <c r="D104" t="s">
-        <v>212</v>
+        <v>219</v>
       </c>
       <c r="E104" t="s">
         <v>46</v>
@@ -2607,16 +2661,16 @@
     </row>
     <row r="105">
       <c r="A105" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="B105" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="C105" t="s">
-        <v>213</v>
+        <v>220</v>
       </c>
       <c r="D105" t="s">
-        <v>212</v>
+        <v>219</v>
       </c>
       <c r="E105" t="s">
         <v>46</v>
@@ -2624,16 +2678,16 @@
     </row>
     <row r="106">
       <c r="A106" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="B106" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="C106" t="s">
-        <v>213</v>
+        <v>220</v>
       </c>
       <c r="D106" t="s">
-        <v>212</v>
+        <v>219</v>
       </c>
       <c r="E106" t="s">
         <v>46</v>
@@ -2641,33 +2695,33 @@
     </row>
     <row r="107">
       <c r="A107" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="B107" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="C107" t="s">
-        <v>252</v>
+        <v>220</v>
       </c>
       <c r="D107" t="s">
-        <v>251</v>
+        <v>219</v>
       </c>
       <c r="E107" t="s">
-        <v>9</v>
+        <v>46</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B108" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="C108" t="s">
-        <v>213</v>
+        <v>220</v>
       </c>
       <c r="D108" t="s">
-        <v>212</v>
+        <v>219</v>
       </c>
       <c r="E108" t="s">
         <v>46</v>
@@ -2675,16 +2729,16 @@
     </row>
     <row r="109">
       <c r="A109" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="B109" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="C109" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="D109" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="E109" t="s">
         <v>9</v>
@@ -2692,32 +2746,44 @@
     </row>
     <row r="110">
       <c r="A110" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="B110" t="s">
-        <v>259</v>
+        <v>261</v>
+      </c>
+      <c r="C110" t="s">
+        <v>220</v>
+      </c>
+      <c r="D110" t="s">
+        <v>219</v>
       </c>
       <c r="E110" t="s">
-        <v>12</v>
+        <v>46</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="B111" t="s">
-        <v>261</v>
+        <v>263</v>
+      </c>
+      <c r="C111" t="s">
+        <v>264</v>
+      </c>
+      <c r="D111" t="s">
+        <v>263</v>
       </c>
       <c r="E111" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="B112" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="E112" t="s">
         <v>12</v>
@@ -2725,10 +2791,10 @@
     </row>
     <row r="113">
       <c r="A113" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="B113" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="E113" t="s">
         <v>12</v>
@@ -2736,64 +2802,58 @@
     </row>
     <row r="114">
       <c r="A114" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="B114" t="s">
-        <v>267</v>
-      </c>
-      <c r="C114" t="s">
-        <v>268</v>
-      </c>
-      <c r="D114" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="E114" t="s">
-        <v>9</v>
-      </c>
-      <c r="F114" t="s">
-        <v>268</v>
+        <v>12</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="B115" t="s">
-        <v>270</v>
-      </c>
-      <c r="C115" t="s">
-        <v>144</v>
-      </c>
-      <c r="D115" t="s">
-        <v>145</v>
+        <v>272</v>
       </c>
       <c r="E115" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="B116" t="s">
-        <v>272</v>
+        <v>274</v>
+      </c>
+      <c r="C116" t="s">
+        <v>275</v>
+      </c>
+      <c r="D116" t="s">
+        <v>274</v>
       </c>
       <c r="E116" t="s">
-        <v>12</v>
+        <v>9</v>
+      </c>
+      <c r="F116" t="s">
+        <v>275</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="B117" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="C117" t="s">
-        <v>275</v>
+        <v>149</v>
       </c>
       <c r="D117" t="s">
-        <v>276</v>
+        <v>150</v>
       </c>
       <c r="E117" t="s">
         <v>9</v>
@@ -2801,50 +2861,44 @@
     </row>
     <row r="118">
       <c r="A118" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B118" t="s">
-        <v>278</v>
-      </c>
-      <c r="C118" t="s">
-        <v>275</v>
-      </c>
-      <c r="D118" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="E118" t="s">
-        <v>81</v>
+        <v>12</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B119" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C119" t="s">
-        <v>275</v>
+        <v>282</v>
       </c>
       <c r="D119" t="s">
-        <v>276</v>
+        <v>283</v>
       </c>
       <c r="E119" t="s">
-        <v>81</v>
+        <v>9</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="B120" t="s">
+        <v>285</v>
+      </c>
+      <c r="C120" t="s">
         <v>282</v>
       </c>
-      <c r="C120" t="s">
-        <v>275</v>
-      </c>
       <c r="D120" t="s">
-        <v>276</v>
+        <v>283</v>
       </c>
       <c r="E120" t="s">
         <v>81</v>
@@ -2852,16 +2906,16 @@
     </row>
     <row r="121">
       <c r="A121" t="s">
+        <v>286</v>
+      </c>
+      <c r="B121" t="s">
+        <v>287</v>
+      </c>
+      <c r="C121" t="s">
+        <v>282</v>
+      </c>
+      <c r="D121" t="s">
         <v>283</v>
-      </c>
-      <c r="B121" t="s">
-        <v>284</v>
-      </c>
-      <c r="C121" t="s">
-        <v>275</v>
-      </c>
-      <c r="D121" t="s">
-        <v>276</v>
       </c>
       <c r="E121" t="s">
         <v>81</v>
@@ -2869,33 +2923,33 @@
     </row>
     <row r="122">
       <c r="A122" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="B122" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="C122" t="s">
-        <v>155</v>
+        <v>282</v>
       </c>
       <c r="D122" t="s">
-        <v>156</v>
+        <v>283</v>
       </c>
       <c r="E122" t="s">
-        <v>9</v>
+        <v>81</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="B123" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="C123" t="s">
-        <v>155</v>
+        <v>282</v>
       </c>
       <c r="D123" t="s">
-        <v>156</v>
+        <v>283</v>
       </c>
       <c r="E123" t="s">
         <v>81</v>
@@ -2903,33 +2957,33 @@
     </row>
     <row r="124">
       <c r="A124" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="B124" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="C124" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="D124" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="E124" t="s">
-        <v>81</v>
+        <v>9</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="B125" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="C125" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="D125" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="E125" t="s">
         <v>81</v>
@@ -2937,16 +2991,16 @@
     </row>
     <row r="126">
       <c r="A126" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="B126" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="C126" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="D126" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="E126" t="s">
         <v>81</v>
@@ -2954,16 +3008,16 @@
     </row>
     <row r="127">
       <c r="A127" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="B127" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="C127" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="D127" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="E127" t="s">
         <v>81</v>
@@ -2971,16 +3025,16 @@
     </row>
     <row r="128">
       <c r="A128" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="B128" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="C128" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="D128" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="E128" t="s">
         <v>81</v>
@@ -2988,16 +3042,16 @@
     </row>
     <row r="129">
       <c r="A129" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="B129" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="C129" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="D129" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="E129" t="s">
         <v>81</v>
@@ -3005,16 +3059,16 @@
     </row>
     <row r="130">
       <c r="A130" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="B130" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="C130" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="D130" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="E130" t="s">
         <v>81</v>
@@ -3022,16 +3076,16 @@
     </row>
     <row r="131">
       <c r="A131" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="B131" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="C131" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="D131" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="E131" t="s">
         <v>81</v>
@@ -3039,83 +3093,95 @@
     </row>
     <row r="132">
       <c r="A132" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="B132" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="C132" t="s">
-        <v>307</v>
+        <v>160</v>
       </c>
       <c r="D132" t="s">
-        <v>306</v>
+        <v>161</v>
       </c>
       <c r="E132" t="s">
-        <v>9</v>
+        <v>81</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="B133" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="C133" t="s">
-        <v>140</v>
+        <v>160</v>
       </c>
       <c r="D133" t="s">
-        <v>141</v>
+        <v>161</v>
       </c>
       <c r="E133" t="s">
-        <v>9</v>
+        <v>81</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="B134" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="C134" t="s">
-        <v>140</v>
+        <v>314</v>
       </c>
       <c r="D134" t="s">
-        <v>141</v>
+        <v>313</v>
       </c>
       <c r="E134" t="s">
-        <v>81</v>
+        <v>9</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="B135" t="s">
-        <v>313</v>
+        <v>316</v>
+      </c>
+      <c r="C135" t="s">
+        <v>145</v>
+      </c>
+      <c r="D135" t="s">
+        <v>146</v>
       </c>
       <c r="E135" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="B136" t="s">
-        <v>315</v>
+        <v>318</v>
+      </c>
+      <c r="C136" t="s">
+        <v>145</v>
+      </c>
+      <c r="D136" t="s">
+        <v>146</v>
       </c>
       <c r="E136" t="s">
-        <v>12</v>
+        <v>81</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="B137" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="E137" t="s">
         <v>12</v>
@@ -3123,13 +3189,80 @@
     </row>
     <row r="138">
       <c r="A138" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="B138" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="E138" t="s">
         <v>12</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="s">
+        <v>323</v>
+      </c>
+      <c r="B139" t="s">
+        <v>324</v>
+      </c>
+      <c r="E139" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="s">
+        <v>325</v>
+      </c>
+      <c r="B140" t="s">
+        <v>326</v>
+      </c>
+      <c r="E140" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="s">
+        <v>327</v>
+      </c>
+      <c r="B141" t="s">
+        <v>328</v>
+      </c>
+      <c r="C141" t="s">
+        <v>329</v>
+      </c>
+      <c r="D141" t="s">
+        <v>330</v>
+      </c>
+      <c r="E141" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="s">
+        <v>331</v>
+      </c>
+      <c r="B142" t="s">
+        <v>332</v>
+      </c>
+      <c r="E142" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="s">
+        <v>333</v>
+      </c>
+      <c r="B143" t="s">
+        <v>334</v>
+      </c>
+      <c r="C143" t="s">
+        <v>335</v>
+      </c>
+      <c r="D143" t="s">
+        <v>336</v>
+      </c>
+      <c r="E143" t="s">
+        <v>136</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refresh generated derivation artifacts (#22)
</commit_message>
<xml_diff>
--- a/crosswalk/FT3-F3-crosswalk.xlsx
+++ b/crosswalk/FT3-F3-crosswalk.xlsx
@@ -8,7 +8,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="320">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="337" uniqueCount="337">
   <si>
     <t>ft3_id</t>
   </si>
@@ -406,6 +406,21 @@
     <t>Phishing: Backup Code</t>
   </si>
   <si>
+    <t>FT016.004</t>
+  </si>
+  <si>
+    <t>Phishing: Real-Time OTP Relay via Operator-Controlled Phishing Kit</t>
+  </si>
+  <si>
+    <t>T1111</t>
+  </si>
+  <si>
+    <t>Multi-Factor Authentication Interception</t>
+  </si>
+  <si>
+    <t>partial</t>
+  </si>
+  <si>
     <t>FT017</t>
   </si>
   <si>
@@ -529,6 +544,12 @@
     <t>Falsifying Business Documents: Fake SS-4 Confirmation Letter</t>
   </si>
   <si>
+    <t>FT026.006</t>
+  </si>
+  <si>
+    <t>Falsifying Business Documents: Live-Source Tax Certificate Forgery</t>
+  </si>
+  <si>
     <t>FT027</t>
   </si>
   <si>
@@ -968,6 +989,36 @@
   </si>
   <si>
     <t>Card Holder Details Collection: Card Details</t>
+  </si>
+  <si>
+    <t>FT057</t>
+  </si>
+  <si>
+    <t>Voice Phishing (Vishing)</t>
+  </si>
+  <si>
+    <t>F1040</t>
+  </si>
+  <si>
+    <t>Phone Number Spoofing</t>
+  </si>
+  <si>
+    <t>FT058</t>
+  </si>
+  <si>
+    <t>ClickFix Run-Dialog Social Engineering</t>
+  </si>
+  <si>
+    <t>FT059</t>
+  </si>
+  <si>
+    <t>Mobile Banking Trojan Distribution and Device Takeover</t>
+  </si>
+  <si>
+    <t>T1453</t>
+  </si>
+  <si>
+    <t>Abuse Accessibility Features</t>
   </si>
 </sst>
 </file>
@@ -1902,7 +1953,7 @@
         <v>135</v>
       </c>
       <c r="E54" t="s">
-        <v>81</v>
+        <v>136</v>
       </c>
       <c r="F54" t="s">
         <v>134</v>
@@ -1910,162 +1961,165 @@
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B55" t="s">
-        <v>137</v>
+        <v>138</v>
+      </c>
+      <c r="C55" t="s">
+        <v>139</v>
+      </c>
+      <c r="D55" t="s">
+        <v>140</v>
       </c>
       <c r="E55" t="s">
-        <v>12</v>
+        <v>81</v>
+      </c>
+      <c r="F55" t="s">
+        <v>139</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="B56" t="s">
-        <v>139</v>
-      </c>
-      <c r="C56" t="s">
-        <v>140</v>
-      </c>
-      <c r="D56" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="E56" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B57" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C57" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D57" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E57" t="s">
-        <v>81</v>
+        <v>9</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B58" t="s">
-        <v>147</v>
+        <v>148</v>
+      </c>
+      <c r="C58" t="s">
+        <v>149</v>
+      </c>
+      <c r="D58" t="s">
+        <v>150</v>
       </c>
       <c r="E58" t="s">
-        <v>12</v>
+        <v>81</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="B59" t="s">
-        <v>149</v>
-      </c>
-      <c r="C59" t="s">
-        <v>150</v>
-      </c>
-      <c r="D59" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="E59" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B60" t="s">
-        <v>152</v>
+        <v>154</v>
+      </c>
+      <c r="C60" t="s">
+        <v>155</v>
+      </c>
+      <c r="D60" t="s">
+        <v>154</v>
       </c>
       <c r="E60" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="B61" t="s">
-        <v>154</v>
-      </c>
-      <c r="C61" t="s">
-        <v>155</v>
-      </c>
-      <c r="D61" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E61" t="s">
-        <v>81</v>
+        <v>12</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B62" t="s">
-        <v>158</v>
+        <v>159</v>
+      </c>
+      <c r="C62" t="s">
+        <v>160</v>
+      </c>
+      <c r="D62" t="s">
+        <v>161</v>
       </c>
       <c r="E62" t="s">
-        <v>12</v>
+        <v>81</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="B63" t="s">
-        <v>160</v>
-      </c>
-      <c r="C63" t="s">
-        <v>161</v>
-      </c>
-      <c r="D63" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E63" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B64" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C64" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="D64" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="E64" t="s">
-        <v>81</v>
+        <v>9</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="B65" t="s">
+        <v>169</v>
+      </c>
+      <c r="C65" t="s">
         <v>166</v>
       </c>
-      <c r="C65" t="s">
-        <v>161</v>
-      </c>
       <c r="D65" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="E65" t="s">
         <v>81</v>
@@ -2073,16 +2127,16 @@
     </row>
     <row r="66">
       <c r="A66" t="s">
+        <v>170</v>
+      </c>
+      <c r="B66" t="s">
+        <v>171</v>
+      </c>
+      <c r="C66" t="s">
+        <v>166</v>
+      </c>
+      <c r="D66" t="s">
         <v>167</v>
-      </c>
-      <c r="B66" t="s">
-        <v>168</v>
-      </c>
-      <c r="C66" t="s">
-        <v>161</v>
-      </c>
-      <c r="D66" t="s">
-        <v>162</v>
       </c>
       <c r="E66" t="s">
         <v>81</v>
@@ -2090,16 +2144,16 @@
     </row>
     <row r="67">
       <c r="A67" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="B67" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="C67" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="D67" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="E67" t="s">
         <v>81</v>
@@ -2107,16 +2161,16 @@
     </row>
     <row r="68">
       <c r="A68" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="B68" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="C68" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="D68" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="E68" t="s">
         <v>81</v>
@@ -2124,32 +2178,44 @@
     </row>
     <row r="69">
       <c r="A69" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="B69" t="s">
-        <v>174</v>
+        <v>177</v>
+      </c>
+      <c r="C69" t="s">
+        <v>166</v>
+      </c>
+      <c r="D69" t="s">
+        <v>167</v>
       </c>
       <c r="E69" t="s">
-        <v>12</v>
+        <v>81</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="B70" t="s">
-        <v>176</v>
+        <v>179</v>
+      </c>
+      <c r="C70" t="s">
+        <v>166</v>
+      </c>
+      <c r="D70" t="s">
+        <v>167</v>
       </c>
       <c r="E70" t="s">
-        <v>12</v>
+        <v>81</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="B71" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="E71" t="s">
         <v>12</v>
@@ -2157,10 +2223,10 @@
     </row>
     <row r="72">
       <c r="A72" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="B72" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="E72" t="s">
         <v>12</v>
@@ -2168,30 +2234,21 @@
     </row>
     <row r="73">
       <c r="A73" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="B73" t="s">
-        <v>182</v>
-      </c>
-      <c r="C73" t="s">
-        <v>125</v>
-      </c>
-      <c r="D73" t="s">
-        <v>124</v>
+        <v>185</v>
       </c>
       <c r="E73" t="s">
-        <v>46</v>
-      </c>
-      <c r="F73" t="s">
-        <v>125</v>
+        <v>12</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="B74" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="E74" t="s">
         <v>12</v>
@@ -2199,36 +2256,33 @@
     </row>
     <row r="75">
       <c r="A75" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="B75" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="C75" t="s">
-        <v>187</v>
+        <v>125</v>
       </c>
       <c r="D75" t="s">
-        <v>186</v>
+        <v>124</v>
       </c>
       <c r="E75" t="s">
-        <v>9</v>
+        <v>46</v>
+      </c>
+      <c r="F75" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B76" t="s">
-        <v>189</v>
-      </c>
-      <c r="C76" t="s">
-        <v>190</v>
-      </c>
-      <c r="D76" t="s">
         <v>191</v>
       </c>
       <c r="E76" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="77">
@@ -2238,22 +2292,28 @@
       <c r="B77" t="s">
         <v>193</v>
       </c>
+      <c r="C77" t="s">
+        <v>194</v>
+      </c>
+      <c r="D77" t="s">
+        <v>193</v>
+      </c>
       <c r="E77" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B78" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C78" t="s">
-        <v>114</v>
+        <v>197</v>
       </c>
       <c r="D78" t="s">
-        <v>115</v>
+        <v>198</v>
       </c>
       <c r="E78" t="s">
         <v>9</v>
@@ -2261,10 +2321,10 @@
     </row>
     <row r="79">
       <c r="A79" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="B79" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="E79" t="s">
         <v>12</v>
@@ -2272,21 +2332,27 @@
     </row>
     <row r="80">
       <c r="A80" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="B80" t="s">
-        <v>199</v>
+        <v>202</v>
+      </c>
+      <c r="C80" t="s">
+        <v>114</v>
+      </c>
+      <c r="D80" t="s">
+        <v>115</v>
       </c>
       <c r="E80" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="B81" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="E81" t="s">
         <v>12</v>
@@ -2294,10 +2360,10 @@
     </row>
     <row r="82">
       <c r="A82" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="B82" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="E82" t="s">
         <v>12</v>
@@ -2305,27 +2371,21 @@
     </row>
     <row r="83">
       <c r="A83" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="B83" t="s">
-        <v>205</v>
-      </c>
-      <c r="C83" t="s">
-        <v>155</v>
-      </c>
-      <c r="D83" t="s">
-        <v>156</v>
+        <v>208</v>
       </c>
       <c r="E83" t="s">
-        <v>81</v>
+        <v>12</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B84" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="E84" t="s">
         <v>12</v>
@@ -2333,21 +2393,27 @@
     </row>
     <row r="85">
       <c r="A85" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="B85" t="s">
-        <v>152</v>
+        <v>212</v>
+      </c>
+      <c r="C85" t="s">
+        <v>160</v>
+      </c>
+      <c r="D85" t="s">
+        <v>161</v>
       </c>
       <c r="E85" t="s">
-        <v>12</v>
+        <v>81</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="B86" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="E86" t="s">
         <v>12</v>
@@ -2355,67 +2421,55 @@
     </row>
     <row r="87">
       <c r="A87" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="B87" t="s">
-        <v>212</v>
-      </c>
-      <c r="C87" t="s">
-        <v>213</v>
-      </c>
-      <c r="D87" t="s">
-        <v>212</v>
+        <v>157</v>
       </c>
       <c r="E87" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B88" t="s">
-        <v>215</v>
-      </c>
-      <c r="C88" t="s">
-        <v>213</v>
-      </c>
-      <c r="D88" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="E88" t="s">
-        <v>46</v>
+        <v>12</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B89" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="C89" t="s">
-        <v>213</v>
+        <v>220</v>
       </c>
       <c r="D89" t="s">
-        <v>212</v>
+        <v>219</v>
       </c>
       <c r="E89" t="s">
-        <v>46</v>
+        <v>9</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="B90" t="s">
+        <v>222</v>
+      </c>
+      <c r="C90" t="s">
+        <v>220</v>
+      </c>
+      <c r="D90" t="s">
         <v>219</v>
-      </c>
-      <c r="C90" t="s">
-        <v>213</v>
-      </c>
-      <c r="D90" t="s">
-        <v>212</v>
       </c>
       <c r="E90" t="s">
         <v>46</v>
@@ -2423,32 +2477,44 @@
     </row>
     <row r="91">
       <c r="A91" t="s">
+        <v>223</v>
+      </c>
+      <c r="B91" t="s">
+        <v>224</v>
+      </c>
+      <c r="C91" t="s">
         <v>220</v>
       </c>
-      <c r="B91" t="s">
-        <v>221</v>
+      <c r="D91" t="s">
+        <v>219</v>
       </c>
       <c r="E91" t="s">
-        <v>12</v>
+        <v>46</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="B92" t="s">
-        <v>223</v>
+        <v>226</v>
+      </c>
+      <c r="C92" t="s">
+        <v>220</v>
+      </c>
+      <c r="D92" t="s">
+        <v>219</v>
       </c>
       <c r="E92" t="s">
-        <v>12</v>
+        <v>46</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="B93" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="E93" t="s">
         <v>12</v>
@@ -2456,10 +2522,10 @@
     </row>
     <row r="94">
       <c r="A94" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="B94" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="E94" t="s">
         <v>12</v>
@@ -2467,10 +2533,10 @@
     </row>
     <row r="95">
       <c r="A95" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="B95" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="E95" t="s">
         <v>12</v>
@@ -2478,10 +2544,10 @@
     </row>
     <row r="96">
       <c r="A96" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="B96" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="E96" t="s">
         <v>12</v>
@@ -2489,10 +2555,10 @@
     </row>
     <row r="97">
       <c r="A97" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="B97" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="E97" t="s">
         <v>12</v>
@@ -2500,10 +2566,10 @@
     </row>
     <row r="98">
       <c r="A98" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="B98" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="E98" t="s">
         <v>12</v>
@@ -2511,10 +2577,10 @@
     </row>
     <row r="99">
       <c r="A99" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="B99" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="E99" t="s">
         <v>12</v>
@@ -2522,67 +2588,55 @@
     </row>
     <row r="100">
       <c r="A100" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="B100" t="s">
-        <v>212</v>
-      </c>
-      <c r="C100" t="s">
-        <v>213</v>
-      </c>
-      <c r="D100" t="s">
-        <v>212</v>
+        <v>242</v>
       </c>
       <c r="E100" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="B101" t="s">
-        <v>240</v>
-      </c>
-      <c r="C101" t="s">
-        <v>213</v>
-      </c>
-      <c r="D101" t="s">
-        <v>212</v>
+        <v>244</v>
       </c>
       <c r="E101" t="s">
-        <v>46</v>
+        <v>12</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="B102" t="s">
         <v>219</v>
       </c>
       <c r="C102" t="s">
-        <v>213</v>
+        <v>220</v>
       </c>
       <c r="D102" t="s">
-        <v>212</v>
+        <v>219</v>
       </c>
       <c r="E102" t="s">
-        <v>46</v>
+        <v>9</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="B103" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="C103" t="s">
-        <v>213</v>
+        <v>220</v>
       </c>
       <c r="D103" t="s">
-        <v>212</v>
+        <v>219</v>
       </c>
       <c r="E103" t="s">
         <v>46</v>
@@ -2590,16 +2644,16 @@
     </row>
     <row r="104">
       <c r="A104" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="B104" t="s">
-        <v>245</v>
+        <v>226</v>
       </c>
       <c r="C104" t="s">
-        <v>213</v>
+        <v>220</v>
       </c>
       <c r="D104" t="s">
-        <v>212</v>
+        <v>219</v>
       </c>
       <c r="E104" t="s">
         <v>46</v>
@@ -2607,16 +2661,16 @@
     </row>
     <row r="105">
       <c r="A105" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="B105" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="C105" t="s">
-        <v>213</v>
+        <v>220</v>
       </c>
       <c r="D105" t="s">
-        <v>212</v>
+        <v>219</v>
       </c>
       <c r="E105" t="s">
         <v>46</v>
@@ -2624,16 +2678,16 @@
     </row>
     <row r="106">
       <c r="A106" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="B106" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="C106" t="s">
-        <v>213</v>
+        <v>220</v>
       </c>
       <c r="D106" t="s">
-        <v>212</v>
+        <v>219</v>
       </c>
       <c r="E106" t="s">
         <v>46</v>
@@ -2641,33 +2695,33 @@
     </row>
     <row r="107">
       <c r="A107" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="B107" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="C107" t="s">
-        <v>252</v>
+        <v>220</v>
       </c>
       <c r="D107" t="s">
-        <v>251</v>
+        <v>219</v>
       </c>
       <c r="E107" t="s">
-        <v>9</v>
+        <v>46</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B108" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="C108" t="s">
-        <v>213</v>
+        <v>220</v>
       </c>
       <c r="D108" t="s">
-        <v>212</v>
+        <v>219</v>
       </c>
       <c r="E108" t="s">
         <v>46</v>
@@ -2675,16 +2729,16 @@
     </row>
     <row r="109">
       <c r="A109" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="B109" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="C109" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="D109" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="E109" t="s">
         <v>9</v>
@@ -2692,32 +2746,44 @@
     </row>
     <row r="110">
       <c r="A110" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="B110" t="s">
-        <v>259</v>
+        <v>261</v>
+      </c>
+      <c r="C110" t="s">
+        <v>220</v>
+      </c>
+      <c r="D110" t="s">
+        <v>219</v>
       </c>
       <c r="E110" t="s">
-        <v>12</v>
+        <v>46</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="B111" t="s">
-        <v>261</v>
+        <v>263</v>
+      </c>
+      <c r="C111" t="s">
+        <v>264</v>
+      </c>
+      <c r="D111" t="s">
+        <v>263</v>
       </c>
       <c r="E111" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="B112" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="E112" t="s">
         <v>12</v>
@@ -2725,10 +2791,10 @@
     </row>
     <row r="113">
       <c r="A113" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="B113" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="E113" t="s">
         <v>12</v>
@@ -2736,64 +2802,58 @@
     </row>
     <row r="114">
       <c r="A114" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="B114" t="s">
-        <v>267</v>
-      </c>
-      <c r="C114" t="s">
-        <v>268</v>
-      </c>
-      <c r="D114" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="E114" t="s">
-        <v>9</v>
-      </c>
-      <c r="F114" t="s">
-        <v>268</v>
+        <v>12</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="B115" t="s">
-        <v>270</v>
-      </c>
-      <c r="C115" t="s">
-        <v>144</v>
-      </c>
-      <c r="D115" t="s">
-        <v>145</v>
+        <v>272</v>
       </c>
       <c r="E115" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="B116" t="s">
-        <v>272</v>
+        <v>274</v>
+      </c>
+      <c r="C116" t="s">
+        <v>275</v>
+      </c>
+      <c r="D116" t="s">
+        <v>274</v>
       </c>
       <c r="E116" t="s">
-        <v>12</v>
+        <v>9</v>
+      </c>
+      <c r="F116" t="s">
+        <v>275</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="B117" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="C117" t="s">
-        <v>275</v>
+        <v>149</v>
       </c>
       <c r="D117" t="s">
-        <v>276</v>
+        <v>150</v>
       </c>
       <c r="E117" t="s">
         <v>9</v>
@@ -2801,50 +2861,44 @@
     </row>
     <row r="118">
       <c r="A118" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B118" t="s">
-        <v>278</v>
-      </c>
-      <c r="C118" t="s">
-        <v>275</v>
-      </c>
-      <c r="D118" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="E118" t="s">
-        <v>81</v>
+        <v>12</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B119" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C119" t="s">
-        <v>275</v>
+        <v>282</v>
       </c>
       <c r="D119" t="s">
-        <v>276</v>
+        <v>283</v>
       </c>
       <c r="E119" t="s">
-        <v>81</v>
+        <v>9</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="B120" t="s">
+        <v>285</v>
+      </c>
+      <c r="C120" t="s">
         <v>282</v>
       </c>
-      <c r="C120" t="s">
-        <v>275</v>
-      </c>
       <c r="D120" t="s">
-        <v>276</v>
+        <v>283</v>
       </c>
       <c r="E120" t="s">
         <v>81</v>
@@ -2852,16 +2906,16 @@
     </row>
     <row r="121">
       <c r="A121" t="s">
+        <v>286</v>
+      </c>
+      <c r="B121" t="s">
+        <v>287</v>
+      </c>
+      <c r="C121" t="s">
+        <v>282</v>
+      </c>
+      <c r="D121" t="s">
         <v>283</v>
-      </c>
-      <c r="B121" t="s">
-        <v>284</v>
-      </c>
-      <c r="C121" t="s">
-        <v>275</v>
-      </c>
-      <c r="D121" t="s">
-        <v>276</v>
       </c>
       <c r="E121" t="s">
         <v>81</v>
@@ -2869,33 +2923,33 @@
     </row>
     <row r="122">
       <c r="A122" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="B122" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="C122" t="s">
-        <v>155</v>
+        <v>282</v>
       </c>
       <c r="D122" t="s">
-        <v>156</v>
+        <v>283</v>
       </c>
       <c r="E122" t="s">
-        <v>9</v>
+        <v>81</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="B123" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="C123" t="s">
-        <v>155</v>
+        <v>282</v>
       </c>
       <c r="D123" t="s">
-        <v>156</v>
+        <v>283</v>
       </c>
       <c r="E123" t="s">
         <v>81</v>
@@ -2903,33 +2957,33 @@
     </row>
     <row r="124">
       <c r="A124" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="B124" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="C124" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="D124" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="E124" t="s">
-        <v>81</v>
+        <v>9</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="B125" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="C125" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="D125" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="E125" t="s">
         <v>81</v>
@@ -2937,16 +2991,16 @@
     </row>
     <row r="126">
       <c r="A126" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="B126" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="C126" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="D126" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="E126" t="s">
         <v>81</v>
@@ -2954,16 +3008,16 @@
     </row>
     <row r="127">
       <c r="A127" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="B127" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="C127" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="D127" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="E127" t="s">
         <v>81</v>
@@ -2971,16 +3025,16 @@
     </row>
     <row r="128">
       <c r="A128" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="B128" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="C128" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="D128" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="E128" t="s">
         <v>81</v>
@@ -2988,16 +3042,16 @@
     </row>
     <row r="129">
       <c r="A129" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="B129" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="C129" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="D129" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="E129" t="s">
         <v>81</v>
@@ -3005,16 +3059,16 @@
     </row>
     <row r="130">
       <c r="A130" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="B130" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="C130" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="D130" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="E130" t="s">
         <v>81</v>
@@ -3022,16 +3076,16 @@
     </row>
     <row r="131">
       <c r="A131" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="B131" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="C131" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="D131" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="E131" t="s">
         <v>81</v>
@@ -3039,83 +3093,95 @@
     </row>
     <row r="132">
       <c r="A132" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="B132" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="C132" t="s">
-        <v>307</v>
+        <v>160</v>
       </c>
       <c r="D132" t="s">
-        <v>306</v>
+        <v>161</v>
       </c>
       <c r="E132" t="s">
-        <v>9</v>
+        <v>81</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="B133" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="C133" t="s">
-        <v>140</v>
+        <v>160</v>
       </c>
       <c r="D133" t="s">
-        <v>141</v>
+        <v>161</v>
       </c>
       <c r="E133" t="s">
-        <v>9</v>
+        <v>81</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="B134" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="C134" t="s">
-        <v>140</v>
+        <v>314</v>
       </c>
       <c r="D134" t="s">
-        <v>141</v>
+        <v>313</v>
       </c>
       <c r="E134" t="s">
-        <v>81</v>
+        <v>9</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="B135" t="s">
-        <v>313</v>
+        <v>316</v>
+      </c>
+      <c r="C135" t="s">
+        <v>145</v>
+      </c>
+      <c r="D135" t="s">
+        <v>146</v>
       </c>
       <c r="E135" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="B136" t="s">
-        <v>315</v>
+        <v>318</v>
+      </c>
+      <c r="C136" t="s">
+        <v>145</v>
+      </c>
+      <c r="D136" t="s">
+        <v>146</v>
       </c>
       <c r="E136" t="s">
-        <v>12</v>
+        <v>81</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="B137" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="E137" t="s">
         <v>12</v>
@@ -3123,13 +3189,80 @@
     </row>
     <row r="138">
       <c r="A138" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="B138" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="E138" t="s">
         <v>12</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="s">
+        <v>323</v>
+      </c>
+      <c r="B139" t="s">
+        <v>324</v>
+      </c>
+      <c r="E139" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="s">
+        <v>325</v>
+      </c>
+      <c r="B140" t="s">
+        <v>326</v>
+      </c>
+      <c r="E140" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="s">
+        <v>327</v>
+      </c>
+      <c r="B141" t="s">
+        <v>328</v>
+      </c>
+      <c r="C141" t="s">
+        <v>329</v>
+      </c>
+      <c r="D141" t="s">
+        <v>330</v>
+      </c>
+      <c r="E141" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="s">
+        <v>331</v>
+      </c>
+      <c r="B142" t="s">
+        <v>332</v>
+      </c>
+      <c r="E142" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="s">
+        <v>333</v>
+      </c>
+      <c r="B143" t="s">
+        <v>334</v>
+      </c>
+      <c r="C143" t="s">
+        <v>335</v>
+      </c>
+      <c r="D143" t="s">
+        <v>336</v>
+      </c>
+      <c r="E143" t="s">
+        <v>136</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refresh derived artifacts for FT060
Automated regen via make publish-ft3 --refresh.
</commit_message>
<xml_diff>
--- a/crosswalk/FT3-F3-crosswalk.xlsx
+++ b/crosswalk/FT3-F3-crosswalk.xlsx
@@ -8,7 +8,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="337" uniqueCount="337">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="339" uniqueCount="339">
   <si>
     <t>ft3_id</t>
   </si>
@@ -1019,6 +1019,12 @@
   </si>
   <si>
     <t>Abuse Accessibility Features</t>
+  </si>
+  <si>
+    <t>FT060</t>
+  </si>
+  <si>
+    <t>Business Email Compromise</t>
   </si>
 </sst>
 </file>
@@ -3265,6 +3271,17 @@
         <v>136</v>
       </c>
     </row>
+    <row r="144">
+      <c r="A144" t="s">
+        <v>337</v>
+      </c>
+      <c r="B144" t="s">
+        <v>338</v>
+      </c>
+      <c r="E144" t="s">
+        <v>12</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>